<commit_message>
Major requirements over time.
</commit_message>
<xml_diff>
--- a/data/classifications/chicago_majors_cip_crosswalk.xlsx
+++ b/data/classifications/chicago_majors_cip_crosswalk.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -15,7 +15,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -279,7 +279,7 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">

</xml_diff>

<commit_message>
choose your own major
</commit_message>
<xml_diff>
--- a/data/classifications/chicago_majors_cip_crosswalk.xlsx
+++ b/data/classifications/chicago_majors_cip_crosswalk.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arijacob/Documents/GitHub/chicago_majors/data/classifications/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21864CC5-D018-A744-92B8-EAFF2450949E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F16263A0-DDC0-E544-A8A5-643EF6583206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="1000" windowWidth="27640" windowHeight="15780" xr2:uid="{2F0C4DB8-871B-E44A-9980-D22782D17142}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="128">
   <si>
     <t>Anthropology</t>
   </si>
@@ -231,13 +231,202 @@
   </si>
   <si>
     <t>guess</t>
+  </si>
+  <si>
+    <t>Comparative Literature</t>
+  </si>
+  <si>
+    <t>Interdisciplinary Studies in the Humanities</t>
+  </si>
+  <si>
+    <t>16.1200</t>
+  </si>
+  <si>
+    <t>05.0200</t>
+  </si>
+  <si>
+    <t>16.0700</t>
+  </si>
+  <si>
+    <t>05.0112</t>
+  </si>
+  <si>
+    <t>16.0400</t>
+  </si>
+  <si>
+    <t>05.0108</t>
+  </si>
+  <si>
+    <t>05.0107</t>
+  </si>
+  <si>
+    <t>05.0299</t>
+  </si>
+  <si>
+    <t>50.0601</t>
+  </si>
+  <si>
+    <t>45.0201</t>
+  </si>
+  <si>
+    <t>27.0101</t>
+  </si>
+  <si>
+    <t>50.0703</t>
+  </si>
+  <si>
+    <t>40.0201</t>
+  </si>
+  <si>
+    <t>40.0599</t>
+  </si>
+  <si>
+    <t>40.0501</t>
+  </si>
+  <si>
+    <t>26.0101</t>
+  </si>
+  <si>
+    <t>16.1299</t>
+  </si>
+  <si>
+    <t>30.2501</t>
+  </si>
+  <si>
+    <t>42.2803</t>
+  </si>
+  <si>
+    <t>11.0299</t>
+  </si>
+  <si>
+    <t>11.0701</t>
+  </si>
+  <si>
+    <t>23.1302</t>
+  </si>
+  <si>
+    <t>30.0601</t>
+  </si>
+  <si>
+    <t>16.0399</t>
+  </si>
+  <si>
+    <t>45.0601</t>
+  </si>
+  <si>
+    <t>45.0603</t>
+  </si>
+  <si>
+    <t>23.0101</t>
+  </si>
+  <si>
+    <t>24.0101</t>
+  </si>
+  <si>
+    <t>40.0603</t>
+  </si>
+  <si>
+    <t>16.0501</t>
+  </si>
+  <si>
+    <t>45.0901</t>
+  </si>
+  <si>
+    <t>54.0104</t>
+  </si>
+  <si>
+    <t>54.0101</t>
+  </si>
+  <si>
+    <t>44.0504</t>
+  </si>
+  <si>
+    <t>38.0206</t>
+  </si>
+  <si>
+    <t>45.9999</t>
+  </si>
+  <si>
+    <t>16.0102</t>
+  </si>
+  <si>
+    <t>9.0702</t>
+  </si>
+  <si>
+    <t>30.1301</t>
+  </si>
+  <si>
+    <t>14.0702</t>
+  </si>
+  <si>
+    <t>50.0901</t>
+  </si>
+  <si>
+    <t>16.1103</t>
+  </si>
+  <si>
+    <t>16.1199</t>
+  </si>
+  <si>
+    <t>26.1501</t>
+  </si>
+  <si>
+    <t>38.0101</t>
+  </si>
+  <si>
+    <t>40.0801</t>
+  </si>
+  <si>
+    <t>45.1001</t>
+  </si>
+  <si>
+    <t>42.0601</t>
+  </si>
+  <si>
+    <t>42.0101</t>
+  </si>
+  <si>
+    <t>42.2704</t>
+  </si>
+  <si>
+    <t>44.0501</t>
+  </si>
+  <si>
+    <t>39.0601</t>
+  </si>
+  <si>
+    <t>16.0999</t>
+  </si>
+  <si>
+    <t>45.1101</t>
+  </si>
+  <si>
+    <t>27.0501</t>
+  </si>
+  <si>
+    <t>50.0507</t>
+  </si>
+  <si>
+    <t>50.0401</t>
+  </si>
+  <si>
+    <t>50.9999</t>
+  </si>
+  <si>
+    <t>16.0104</t>
+  </si>
+  <si>
+    <t>24.0103</t>
+  </si>
+  <si>
+    <t>03.0103</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -253,6 +442,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FF4D4D4C"/>
+      <name val="Lucida Grande"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Lucida Grande"/>
       <family val="2"/>
     </font>
@@ -277,10 +473,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -615,7 +814,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7972D36-0D3F-4C4C-BA70-DBA0E5169024}">
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.1640625" customWidth="1"/>
@@ -640,8 +839,8 @@
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2">
-        <v>45.020099999999999</v>
+      <c r="C2" s="4" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -651,8 +850,8 @@
       <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="2">
-        <v>27.010100000000001</v>
+      <c r="C3" s="4" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -662,8 +861,8 @@
       <c r="B4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="2">
-        <v>50.070300000000003</v>
+      <c r="C4" s="4" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -673,8 +872,8 @@
       <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="2">
-        <v>40.020099999999999</v>
+      <c r="C5" s="4" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -684,8 +883,8 @@
       <c r="B6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="2">
-        <v>40.059899999999999</v>
+      <c r="C6" s="4" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -695,8 +894,8 @@
       <c r="B7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="2">
-        <v>26.010100000000001</v>
+      <c r="C7" s="4" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -706,8 +905,8 @@
       <c r="B8" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="2">
-        <v>40.0501</v>
+      <c r="C8" s="4" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -717,8 +916,8 @@
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="2">
-        <v>50.060099999999998</v>
+      <c r="C9" s="4" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -728,541 +927,665 @@
       <c r="B10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="2">
-        <v>16.12</v>
+      <c r="C10" s="4" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="2">
-        <v>30.2501</v>
-      </c>
+      <c r="C11" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D11" s="2"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C12" s="2">
-        <v>42.280299999999997</v>
-      </c>
-      <c r="D12" t="s">
-        <v>64</v>
+        <v>5</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C13" s="2">
-        <v>27.010100000000001</v>
+        <v>1</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D13" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C14" s="2">
-        <v>11.0701</v>
+      <c r="C14" s="4" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C15" s="2">
-        <v>23.130199999999999</v>
+        <v>3</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C17" s="2">
-        <v>30.060099999999998</v>
+        <v>5</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C18" s="2">
-        <v>16.039899999999999</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="C18" s="5"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C19" s="2">
-        <v>45.060299999999998</v>
+        <v>3</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C20" s="2">
-        <v>23.010100000000001</v>
+      <c r="C20" s="4" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C21" s="2">
-        <v>45.070099999999996</v>
+      <c r="C21" s="4" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C22" s="2">
-        <v>3.0103</v>
+        <v>1</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C23" s="2">
-        <v>3.0103</v>
+        <v>5</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C24" s="2">
-        <v>24.010100000000001</v>
-      </c>
-      <c r="D24" t="s">
-        <v>64</v>
+        <v>1</v>
+      </c>
+      <c r="C24" s="4">
+        <v>45.070099999999996</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C25" s="2">
-        <v>5.0298999999999996</v>
-      </c>
-      <c r="D25" s="2"/>
+        <v>3</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C26" s="2">
-        <v>40.060299999999998</v>
+        <v>1</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C27" s="2">
-        <v>16.0501</v>
+      <c r="C27" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D27" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C28" s="2">
-        <v>45.0901</v>
-      </c>
-      <c r="D28" t="s">
-        <v>64</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D28" s="2"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C29" s="2">
-        <v>54.010399999999997</v>
+        <v>3</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C30" s="2">
-        <v>54.010100000000001</v>
+        <v>5</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C31" s="2">
-        <v>44.050400000000003</v>
+      <c r="C31" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="D31" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="1" t="s">
+      <c r="B35" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C35" s="5"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C33" s="2">
-        <v>38.020600000000002</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="1" t="s">
+      <c r="B36" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C34" s="2">
-        <v>5.0106999999999999</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="1" t="s">
+      <c r="B37" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C35" s="2">
-        <v>45.999899999999997</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="1" t="s">
+      <c r="B38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C36" s="2">
-        <v>16.010200000000001</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" s="1" t="s">
+      <c r="B39" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C37" s="2">
-        <v>27.010100000000001</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C38" s="2">
-        <v>9.0701999999999998</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C39" s="2">
-        <v>30.130099999999999</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C40" s="2">
-        <v>14.0702</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="C40" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B41" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C41" s="2">
-        <v>50.0901</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="1" t="s">
+      <c r="B44" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B42" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C42" s="2">
-        <v>16.119900000000001</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A43" s="1" t="s">
+      <c r="B45" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="B48" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C43" s="2">
-        <v>26.150099999999998</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A44" s="1" t="s">
+      <c r="C48" s="4" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B44" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C44" s="2">
-        <v>38.010100000000001</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="1" t="s">
+      <c r="B49" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B45" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C45" s="2">
-        <v>38.010100000000001</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="1" t="s">
+      <c r="B50" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B51" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C46" s="2">
-        <v>40.080100000000002</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="1" t="s">
+      <c r="C51" s="4" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B47" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C47" s="2">
-        <v>45.100099999999998</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" s="1" t="s">
+      <c r="B52" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B48" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C48" s="2">
-        <v>42.270400000000002</v>
-      </c>
-      <c r="D48" s="2"/>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A49" s="1" t="s">
+      <c r="B53" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B49" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C49" s="2">
-        <v>44.0501</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A50" s="1" t="s">
+      <c r="B56" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B50" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C50" s="2">
-        <v>5.0199999999999996</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A51" s="1" t="s">
+      <c r="B57" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B51" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C51" s="2">
-        <v>39.060099999999998</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A52" s="1" t="s">
+      <c r="B58" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A59" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B52" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C52" s="2">
-        <v>16.099900000000002</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A53" s="1" t="s">
+      <c r="B59" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A60" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B53" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C53" s="2">
-        <v>16.04</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A54" s="1" t="s">
+      <c r="B60" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B54" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C54" s="2">
-        <v>45.110100000000003</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A55" s="1" t="s">
+      <c r="B61" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B55" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C55" s="2">
-        <v>16.07</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A56" s="1" t="s">
+      <c r="B62" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D63" s="3"/>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B64" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C56" s="2">
-        <v>27.0501</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A57" s="1" t="s">
+      <c r="C64" s="4" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B57" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C57" s="2">
-        <v>50.050699999999999</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A58" s="1" t="s">
+      <c r="B65" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B58" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C58" s="2">
-        <v>50.999899999999997</v>
+      <c r="B66" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>66</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>